<commit_message>
Update IT23668768.xlsx with latest test automation data
</commit_message>
<xml_diff>
--- a/IT23668768/test_automation/test_automation/IT23668768.xlsx
+++ b/IT23668768/test_automation/test_automation/IT23668768.xlsx
@@ -1595,7 +1595,7 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t>මම 3 ඩෙනට කන්න ගෙන එන්නම්.</t>
+          <t>අපි 10 මිනිට් පස්සෙ යනwඅ.</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -2309,7 +2309,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>මෙක මර සෙට් එකක් බ්‍රො.</t>
+          <t>මෙ බග් එක ක්ග් 10ක් wඉතර.</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>සිරwඅටම එය cලස්ස් කිwwඅ.</t>
+          <t>මෙ බග් එක ක්ග් 10ක් wඉතර.</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
@@ -2393,7 +2393,7 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>මෙ ලින්ක් එක බලල: www.ගෝග්ලෙ.cඔම් මම මෙක උසෙ කරනwඅ.</t>
+          <t>මෙ බග් එක ක්ග් 10ක් wඉතර.</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>@ඛසුන් අය්ය ඔය ෆ්‍රේ ඩ පොඩ්ඩක් cඅල්ල් කරන්න.</t>
+          <t>මෙ බග් එක ක්ග් 10ක් wඉතර.</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>මම ටිරෙඩ් wඑල 😩 ගෙඩර යනwඅ.</t>
+          <t>මෙ බග් එක ක්ග් 10ක් wඉතර.</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>එය මෙක කරල 😂 මම ඩන්නwඅ නේ.</t>
+          <t>මෙ බග් එක ක්ග් 10ක් wඉතර.</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>ඔය 5pm ට ඔෆ්ෆිcඑ එකෙන් යනwඅ ඩ, නට්ටම් 6pm ට?</t>
+          <t>මෙ බග් එක ක්ග් 10ක් wඉතර.</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>මචන් මෙක මර ඉස්සුඑ එකක් 😤 අසප් බලන්න, නට්ටම් අපි ලටෙ wඑයි.</t>
+          <t>මෙ බග් එක ක්ග් 10ක් wඉතර.</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Rename test automation script and update README references
</commit_message>
<xml_diff>
--- a/IT23668768/test_automation/test_automation/IT23668768.xlsx
+++ b/IT23668768/test_automation/test_automation/IT23668768.xlsx
@@ -2309,7 +2309,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>මෙ බග් එක ක්ග් 10ක් wඉතර.</t>
+          <t>මෙක මර සෙට් එකක් බ්‍රො.</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
@@ -2351,7 +2351,7 @@
       </c>
       <c r="E45" s="5" t="inlineStr">
         <is>
-          <t>මෙ බග් එක ක්ග් 10ක් wඉතර.</t>
+          <t>සිරwඅටම එය cලස්ස් කිwwඅ.</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
@@ -2393,7 +2393,7 @@
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>මෙ බග් එක ක්ග් 10ක් wඉතර.</t>
+          <t>මෙ ලින්ක් එක බලල: www.ගෝග්ලෙ.cඔම් මම මෙක උසෙ කරනwඅ.</t>
         </is>
       </c>
       <c r="F46" s="3" t="inlineStr">
@@ -2435,7 +2435,7 @@
       </c>
       <c r="E47" s="5" t="inlineStr">
         <is>
-          <t>මෙ බග් එක ක්ග් 10ක් wඉතර.</t>
+          <t>@ඛසුන් අය්ය ඔය ෆ්‍රේ ඩ පොඩ්ඩක් cඅල්ල් කරන්න.</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
@@ -2477,7 +2477,7 @@
       </c>
       <c r="E48" s="3" t="inlineStr">
         <is>
-          <t>මෙ බග් එක ක්ග් 10ක් wඉතර.</t>
+          <t>මම ටිරෙඩ් wඑල 😩 ගෙඩර යනwඅ.</t>
         </is>
       </c>
       <c r="F48" s="3" t="inlineStr">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr">
         <is>
-          <t>මෙ බග් එක ක්ග් 10ක් wඉතර.</t>
+          <t>එය මෙක කරල 😂 මම ඩන්නwඅ නේ.</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
@@ -2561,7 +2561,7 @@
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>මෙ බග් එක ක්ග් 10ක් wඉතර.</t>
+          <t>ඔය 5pm ට ඔෆ්ෆිcඑ එකෙන් යනwඅ ඩ, නට්ටම් 6pm ට?</t>
         </is>
       </c>
       <c r="F50" s="3" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>මෙ බග් එක ක්ග් 10ක් wඉතර.</t>
+          <t>මචන් මෙක මර ඉස්සුඑ එකක් 😤 අසප් බලන්න, නට්ටම් අපි ලටෙ wඑයි.</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">

</xml_diff>